<commit_message>
build: rebuild module artifacts
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/IpAddressConditionalFormattingTemplate.xlsx
+++ b/Data/IpAddressConditionalFormattingTemplate.xlsx
@@ -195,7 +195,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="465">
+  <dxfs count="495">
     <dxf>
       <fill>
         <patternFill>
@@ -262,6 +262,216 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
     <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <fill>
         <patternFill>
@@ -3944,31 +4154,31 @@
     <row r="78" ht="15" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="A:A">
-    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="460">
+    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="490">
       <formula>NOT(ISERROR(SEARCH("microsoft",A1)))</formula>
     </cfRule>
-    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="461">
+    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="491">
       <formula>NOT(ISERROR(SEARCH("proofpoint",A1)))</formula>
     </cfRule>
-    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="462">
+    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="492">
       <formula>NOT(ISERROR(SEARCH(" vpn",A1)))</formula>
     </cfRule>
-    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="462">
+    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="492">
       <formula>NOT(ISERROR(SEARCH(" tor",A1)))</formula>
     </cfRule>
-    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="462">
+    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="492">
       <formula>NOT(ISERROR(SEARCH(" proxy",A1)))</formula>
     </cfRule>
-    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="463">
+    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="493">
       <formula>NOT(ISERROR(SEARCH(" hosting",A1)))</formula>
     </cfRule>
-    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="463">
+    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="493">
       <formula>NOT(ISERROR(SEARCH(" cloud",A1)))</formula>
     </cfRule>
-    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="463">
+    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="493">
       <formula>NOT(ISERROR(SEARCH(" datacenter",A1)))</formula>
     </cfRule>
-    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="464">
+    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="494">
       <formula>NOT(ISERROR(SEARCH("mobile",A1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>